<commit_message>
Recalculate calendar, budget and plan with Sara's selected ideas (13 videos, 5 carousels, 8 story sets)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FV7y6XEE3x9ogCMyfe3pnd
</commit_message>
<xml_diff>
--- a/docs/sesion-2026-10-02/presupuesto-contenido-oct-dic.xlsx
+++ b/docs/sesion-2026-10-02/presupuesto-contenido-oct-dic.xlsx
@@ -495,12 +495,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C38"/>
+  <dimension ref="A1:C36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="56" customWidth="1" min="1" max="1"/>
+    <col width="58" customWidth="1" min="1" max="1"/>
     <col width="18" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -547,7 +546,7 @@
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>Set de historias (tarifa anterior, CONFIRMAR)</t>
+          <t>Set de historias (por confirmar)</t>
         </is>
       </c>
       <c r="B7" s="5" t="n">
@@ -568,7 +567,7 @@
         </is>
       </c>
       <c r="B10" s="6">
-        <f>COUNTIFS(Calendario!$E$2:$E$48,"Video",Calendario!$F$2:$F$48,"Núcleo")</f>
+        <f>COUNTIFS(Calendario!$F$2:$F$53,"Video",Calendario!$G$2:$G$53,"Núcleo")</f>
         <v/>
       </c>
     </row>
@@ -579,18 +578,18 @@
         </is>
       </c>
       <c r="B11" s="6">
-        <f>COUNTIFS(Calendario!$E$2:$E$48,"Carrusel",Calendario!$F$2:$F$48,"Núcleo")</f>
+        <f>COUNTIFS(Calendario!$F$2:$F$53,"Carrusel",Calendario!$G$2:$G$53,"Núcleo")</f>
         <v/>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
         <is>
-          <t>Sets de historias (opcional)</t>
+          <t>Sets de historias · Núcleo</t>
         </is>
       </c>
       <c r="B12" s="6">
-        <f>COUNTIFS(Calendario!$E$2:$E$48,"Historias")</f>
+        <f>COUNTIFS(Calendario!$F$2:$F$53,"Historias",Calendario!$G$2:$G$53,"Núcleo")</f>
         <v/>
       </c>
     </row>
@@ -601,7 +600,7 @@
         </is>
       </c>
       <c r="B13" s="6">
-        <f>COUNTIFS(Calendario!$F$2:$F$48,"Fase B")</f>
+        <f>COUNTIFS(Calendario!$G$2:$G$53,"Fase B")</f>
         <v/>
       </c>
     </row>
@@ -619,7 +618,7 @@
         </is>
       </c>
       <c r="B16" s="7">
-        <f>SUMIFS(Calendario!$H$2:$H$48,Calendario!$F$2:$F$48,"Núcleo",Calendario!$G$2:$G$48,"A")</f>
+        <f>SUMIFS(Calendario!$I$2:$I$53,Calendario!$G$2:$G$53,"Núcleo",Calendario!$H$2:$H$53,"A")</f>
         <v/>
       </c>
     </row>
@@ -630,7 +629,7 @@
         </is>
       </c>
       <c r="B17" s="7">
-        <f>SUMIFS(Calendario!$H$2:$H$48,Calendario!$F$2:$F$48,"Núcleo",Calendario!$G$2:$G$48,"B")</f>
+        <f>SUMIFS(Calendario!$I$2:$I$53,Calendario!$G$2:$G$53,"Núcleo",Calendario!$H$2:$H$53,"B")</f>
         <v/>
       </c>
     </row>
@@ -648,7 +647,7 @@
     <row r="19">
       <c r="A19" s="8" t="inlineStr">
         <is>
-          <t>OPCIÓN 2 · Completo (núcleo A + B)</t>
+          <t>OPCIÓN 2 · Completo (A + B)</t>
         </is>
       </c>
       <c r="B19" s="9">
@@ -663,7 +662,7 @@
         </is>
       </c>
       <c r="B20" s="7">
-        <f>SUMIFS(Calendario!$H$2:$H$48,Calendario!$F$2:$F$48,"Fase B")</f>
+        <f>SUMIFS(Calendario!$I$2:$I$53,Calendario!$G$2:$G$53,"Fase B")</f>
         <v/>
       </c>
     </row>
@@ -678,138 +677,116 @@
         <v/>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" s="4" t="inlineStr">
-        <is>
-          <t>Historias (opcional)</t>
-        </is>
-      </c>
-      <c r="B22" s="7">
-        <f>SUMIFS(Calendario!$H$2:$H$48,Calendario!$F$2:$F$48,"Historias (opcional)")</f>
-        <v/>
-      </c>
-    </row>
     <row r="23">
-      <c r="A23" s="8" t="inlineStr">
-        <is>
-          <t>OPCIÓN 4 · Todo incluido</t>
-        </is>
-      </c>
-      <c r="B23" s="9">
-        <f>B21+B22</f>
-        <v/>
+      <c r="A23" s="3" t="inlineStr">
+        <is>
+          <t>GASTOS REEMBOLSABLES (ESTIMADOS — confirmar; $0 si Alado ya lo tiene)</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>Luz LED portátil (el taller tiene poca luz)</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="n">
+        <v>180000</v>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="3" t="inlineStr">
-        <is>
-          <t>GASTOS REEMBOLSABLES (ESTIMADOS — confirmar; $0 si Alado ya lo tiene)</t>
-        </is>
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>Micrófono de solapa</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="n">
+        <v>90000</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="4" t="inlineStr">
         <is>
-          <t>Luz LED portátil (el taller tiene poca luz)</t>
+          <t>Trípode / soporte para celular</t>
         </is>
       </c>
       <c r="B26" s="5" t="n">
-        <v>180000</v>
+        <v>70000</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="4" t="inlineStr">
         <is>
-          <t>Micrófono de solapa (voz en off de Alejo)</t>
+          <t>Banco de música con licencia comercial (2 meses)</t>
         </is>
       </c>
       <c r="B27" s="5" t="n">
-        <v>90000</v>
+        <v>100000</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="4" t="inlineStr">
         <is>
-          <t>Trípode / soporte para celular</t>
+          <t>Transporte a El Retiro (4 viajes × $50.000)</t>
         </is>
       </c>
       <c r="B28" s="5" t="n">
-        <v>70000</v>
+        <v>200000</v>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="4" t="inlineStr">
-        <is>
-          <t>Banco de música con licencia comercial (2 meses)</t>
-        </is>
-      </c>
-      <c r="B29" s="5" t="n">
-        <v>100000</v>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="4" t="inlineStr">
-        <is>
-          <t>Transporte a El Retiro (4 viajes × $50.000)</t>
-        </is>
-      </c>
-      <c r="B30" s="5" t="n">
-        <v>200000</v>
+      <c r="A29" s="8" t="inlineStr">
+        <is>
+          <t>Total reembolsables</t>
+        </is>
+      </c>
+      <c r="B29" s="10">
+        <f>SUM(B24:B28)</f>
+        <v/>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="8" t="inlineStr">
-        <is>
-          <t>Total reembolsables</t>
-        </is>
-      </c>
-      <c r="B31" s="10">
-        <f>SUM(B26:B30)</f>
+      <c r="A31" s="3" t="inlineStr">
+        <is>
+          <t>NÚCLEO POR MES (prioridad A + B)</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="inlineStr">
+        <is>
+          <t>Octubre</t>
+        </is>
+      </c>
+      <c r="B32" s="7">
+        <f>SUMIFS(Calendario!$I$2:$I$53,Calendario!$G$2:$G$53,"Núcleo",Calendario!$B$2:$B$53,"&gt;="&amp;DATE(2026,10,1),Calendario!$B$2:$B$53,"&lt;"&amp;DATE(2026,11,1))</f>
         <v/>
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="3" t="inlineStr">
-        <is>
-          <t>NÚCLEO POR MES (prioridad A + B)</t>
-        </is>
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t>Noviembre</t>
+        </is>
+      </c>
+      <c r="B33" s="7">
+        <f>SUMIFS(Calendario!$I$2:$I$53,Calendario!$G$2:$G$53,"Núcleo",Calendario!$B$2:$B$53,"&gt;="&amp;DATE(2026,11,1),Calendario!$B$2:$B$53,"&lt;"&amp;DATE(2026,12,1))</f>
+        <v/>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="4" t="inlineStr">
         <is>
-          <t>Octubre</t>
+          <t>Diciembre</t>
         </is>
       </c>
       <c r="B34" s="7">
-        <f>SUMIFS(Calendario!$H$2:$H$48,Calendario!$F$2:$F$48,"Núcleo",Calendario!$B$2:$B$48,"&gt;="&amp;DATE(2026,10,1),Calendario!$B$2:$B$48,"&lt;"&amp;DATE(2026,11,1))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="4" t="inlineStr">
-        <is>
-          <t>Noviembre</t>
-        </is>
-      </c>
-      <c r="B35" s="7">
-        <f>SUMIFS(Calendario!$H$2:$H$48,Calendario!$F$2:$F$48,"Núcleo",Calendario!$B$2:$B$48,"&gt;="&amp;DATE(2026,11,1),Calendario!$B$2:$B$48,"&lt;"&amp;DATE(2026,12,1))</f>
+        <f>SUMIFS(Calendario!$I$2:$I$53,Calendario!$G$2:$G$53,"Núcleo",Calendario!$B$2:$B$53,"&gt;="&amp;DATE(2026,12,1),Calendario!$B$2:$B$53,"&lt;"&amp;DATE(2027,1,1))</f>
         <v/>
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="4" t="inlineStr">
-        <is>
-          <t>Diciembre</t>
-        </is>
-      </c>
-      <c r="B36" s="7">
-        <f>SUMIFS(Calendario!$H$2:$H$48,Calendario!$F$2:$F$48,"Núcleo",Calendario!$B$2:$B$48,"&gt;="&amp;DATE(2026,12,1),Calendario!$B$2:$B$48,"&lt;"&amp;DATE(2027,1,1))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="2" t="inlineStr">
+      <c r="A36" s="2" t="inlineStr">
         <is>
           <t>Propuesta de pago: 50% al aprobar el plan, 50% contra entrega por mes. Los derechos del contenido son de Alado; Sara puede mostrarlo en su portafolio.</t>
         </is>
@@ -817,9 +794,9 @@
     </row>
   </sheetData>
   <mergeCells count="7">
-    <mergeCell ref="A25:C25"/>
-    <mergeCell ref="A33:C33"/>
     <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A23:C23"/>
+    <mergeCell ref="A31:C31"/>
     <mergeCell ref="A9:C9"/>
     <mergeCell ref="A15:C15"/>
     <mergeCell ref="A4:C4"/>
@@ -835,17 +812,18 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H30"/>
+  <dimension ref="A1:I35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="50" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="22" customWidth="1" min="6" max="6"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="52" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
     <col width="10" customWidth="1" min="7" max="7"/>
-    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="10" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -856,35 +834,40 @@
       </c>
       <c r="B1" s="11" t="inlineStr">
         <is>
-          <t>Fecha</t>
+          <t>Publica</t>
         </is>
       </c>
       <c r="C1" s="11" t="inlineStr">
         <is>
+          <t>Se graba</t>
+        </is>
+      </c>
+      <c r="D1" s="11" t="inlineStr">
+        <is>
           <t>Línea</t>
         </is>
       </c>
-      <c r="D1" s="11" t="inlineStr">
+      <c r="E1" s="11" t="inlineStr">
         <is>
           <t>Pieza</t>
         </is>
       </c>
-      <c r="E1" s="11" t="inlineStr">
+      <c r="F1" s="11" t="inlineStr">
         <is>
           <t>Formato</t>
         </is>
       </c>
-      <c r="F1" s="11" t="inlineStr">
+      <c r="G1" s="11" t="inlineStr">
         <is>
           <t>Fase</t>
         </is>
       </c>
-      <c r="G1" s="11" t="inlineStr">
+      <c r="H1" s="11" t="inlineStr">
         <is>
           <t>Prioridad</t>
         </is>
       </c>
-      <c r="H1" s="11" t="inlineStr">
+      <c r="I1" s="11" t="inlineStr">
         <is>
           <t>Valor</t>
         </is>
@@ -893,1072 +876,1427 @@
     <row r="2">
       <c r="A2" s="12" t="inlineStr">
         <is>
-          <t>P01</t>
+          <t>01</t>
         </is>
       </c>
       <c r="B2" s="13" t="n">
-        <v>46301</v>
+        <v>46303</v>
       </c>
       <c r="C2" s="14" t="inlineStr">
         <is>
-          <t>Bride</t>
+          <t>mar 6 oct · pre-taller</t>
         </is>
       </c>
       <c r="D2" s="14" t="inlineStr">
         <is>
-          <t>Así se diseña un vestido en Alado</t>
+          <t>Alado &amp; Co.</t>
         </is>
       </c>
       <c r="E2" s="14" t="inlineStr">
         <is>
-          <t>Carrusel</t>
+          <t>Invitación al taller de cerámica (17 oct)</t>
         </is>
       </c>
       <c r="F2" s="14" t="inlineStr">
         <is>
-          <t>Núcleo</t>
+          <t>Video</t>
         </is>
       </c>
       <c r="G2" s="14" t="inlineStr">
         <is>
+          <t>Núcleo</t>
+        </is>
+      </c>
+      <c r="H2" s="14" t="inlineStr">
+        <is>
           <t>A</t>
         </is>
       </c>
-      <c r="H2" s="7">
-        <f>IF(E2="Video",Presupuesto!$B$5,IF(E2="Carrusel",Presupuesto!$B$6,IF(E2="Historias",Presupuesto!$B$7,0)))</f>
+      <c r="I2" s="7">
+        <f>IF(F2="Video",Presupuesto!$B$5,IF(F2="Carrusel",Presupuesto!$B$6,IF(F2="Historias",Presupuesto!$B$7,0)))</f>
         <v/>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="12" t="inlineStr">
         <is>
-          <t>P02</t>
+          <t>02</t>
         </is>
       </c>
       <c r="B3" s="13" t="n">
-        <v>46303</v>
+        <v>46304</v>
       </c>
       <c r="C3" s="14" t="inlineStr">
         <is>
-          <t>Alado &amp; Co.</t>
+          <t>lun 5 oct · atelier</t>
         </is>
       </c>
       <c r="D3" s="14" t="inlineStr">
         <is>
-          <t>Invitación al taller de cerámica (17 oct)</t>
+          <t>Bride</t>
         </is>
       </c>
       <c r="E3" s="14" t="inlineStr">
         <is>
-          <t>Video</t>
+          <t>B16 · Destacado fijo «Bride» (10 historias)</t>
         </is>
       </c>
       <c r="F3" s="14" t="inlineStr">
         <is>
-          <t>Núcleo</t>
+          <t>Historias</t>
         </is>
       </c>
       <c r="G3" s="14" t="inlineStr">
         <is>
+          <t>Núcleo</t>
+        </is>
+      </c>
+      <c r="H3" s="14" t="inlineStr">
+        <is>
           <t>A</t>
         </is>
       </c>
-      <c r="H3" s="7">
-        <f>IF(E3="Video",Presupuesto!$B$5,IF(E3="Carrusel",Presupuesto!$B$6,IF(E3="Historias",Presupuesto!$B$7,0)))</f>
+      <c r="I3" s="7">
+        <f>IF(F3="Video",Presupuesto!$B$5,IF(F3="Carrusel",Presupuesto!$B$6,IF(F3="Historias",Presupuesto!$B$7,0)))</f>
         <v/>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="12" t="inlineStr">
         <is>
-          <t>P03</t>
+          <t>03</t>
         </is>
       </c>
       <c r="B4" s="13" t="n">
-        <v>46308</v>
+        <v>46307</v>
       </c>
       <c r="C4" s="14" t="inlineStr">
         <is>
-          <t>Bride</t>
+          <t>material existente</t>
         </is>
       </c>
       <c r="D4" s="14" t="inlineStr">
         <is>
-          <t>El figurín en vivo</t>
+          <t>Alado</t>
         </is>
       </c>
       <c r="E4" s="14" t="inlineStr">
         <is>
-          <t>Video</t>
+          <t>A18 · Cómo comprar (Destacado)</t>
         </is>
       </c>
       <c r="F4" s="14" t="inlineStr">
         <is>
-          <t>Núcleo</t>
+          <t>Historias</t>
         </is>
       </c>
       <c r="G4" s="14" t="inlineStr">
         <is>
+          <t>Núcleo</t>
+        </is>
+      </c>
+      <c r="H4" s="14" t="inlineStr">
+        <is>
           <t>A</t>
         </is>
       </c>
-      <c r="H4" s="7">
-        <f>IF(E4="Video",Presupuesto!$B$5,IF(E4="Carrusel",Presupuesto!$B$6,IF(E4="Historias",Presupuesto!$B$7,0)))</f>
+      <c r="I4" s="7">
+        <f>IF(F4="Video",Presupuesto!$B$5,IF(F4="Carrusel",Presupuesto!$B$6,IF(F4="Historias",Presupuesto!$B$7,0)))</f>
         <v/>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="12" t="inlineStr">
         <is>
-          <t>P04</t>
+          <t>04</t>
         </is>
       </c>
       <c r="B5" s="13" t="n">
-        <v>46315</v>
+        <v>46308</v>
       </c>
       <c r="C5" s="14" t="inlineStr">
         <is>
-          <t>Alado &amp; Co.</t>
+          <t>lun 5 oct · atelier</t>
         </is>
       </c>
       <c r="D5" s="14" t="inlineStr">
         <is>
-          <t>Recap del taller de cerámica</t>
+          <t>Bride</t>
         </is>
       </c>
       <c r="E5" s="14" t="inlineStr">
         <is>
+          <t>B1 · El figurín en vivo</t>
+        </is>
+      </c>
+      <c r="F5" s="14" t="inlineStr">
+        <is>
           <t>Video</t>
         </is>
       </c>
-      <c r="F5" s="14" t="inlineStr">
-        <is>
-          <t>Núcleo</t>
-        </is>
-      </c>
       <c r="G5" s="14" t="inlineStr">
         <is>
+          <t>Núcleo</t>
+        </is>
+      </c>
+      <c r="H5" s="14" t="inlineStr">
+        <is>
           <t>A</t>
         </is>
       </c>
-      <c r="H5" s="7">
-        <f>IF(E5="Video",Presupuesto!$B$5,IF(E5="Carrusel",Presupuesto!$B$6,IF(E5="Historias",Presupuesto!$B$7,0)))</f>
+      <c r="I5" s="7">
+        <f>IF(F5="Video",Presupuesto!$B$5,IF(F5="Carrusel",Presupuesto!$B$6,IF(F5="Historias",Presupuesto!$B$7,0)))</f>
         <v/>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="12" t="inlineStr">
         <is>
-          <t>P05</t>
+          <t>05</t>
         </is>
       </c>
       <c r="B6" s="13" t="n">
-        <v>46317</v>
+        <v>46309</v>
       </c>
       <c r="C6" s="14" t="inlineStr">
         <is>
-          <t>Alado (ropa)</t>
+          <t>mar 6 oct y sáb 17 oct</t>
         </is>
       </c>
       <c r="D6" s="14" t="inlineStr">
         <is>
-          <t>Una pieza, su historia</t>
+          <t>Alado &amp; Co.</t>
         </is>
       </c>
       <c r="E6" s="14" t="inlineStr">
         <is>
-          <t>Carrusel</t>
+          <t>C18 · Taller: cupos, cuenta regresiva y en vivo</t>
         </is>
       </c>
       <c r="F6" s="14" t="inlineStr">
         <is>
-          <t>Núcleo</t>
+          <t>Historias</t>
         </is>
       </c>
       <c r="G6" s="14" t="inlineStr">
         <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="H6" s="7">
-        <f>IF(E6="Video",Presupuesto!$B$5,IF(E6="Carrusel",Presupuesto!$B$6,IF(E6="Historias",Presupuesto!$B$7,0)))</f>
+          <t>Núcleo</t>
+        </is>
+      </c>
+      <c r="H6" s="14" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="I6" s="7">
+        <f>IF(F6="Video",Presupuesto!$B$5,IF(F6="Carrusel",Presupuesto!$B$6,IF(F6="Historias",Presupuesto!$B$7,0)))</f>
         <v/>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="12" t="inlineStr">
         <is>
-          <t>P06</t>
+          <t>06</t>
         </is>
       </c>
       <c r="B7" s="13" t="n">
-        <v>46319</v>
+        <v>46315</v>
       </c>
       <c r="C7" s="14" t="inlineStr">
         <is>
+          <t>sáb 17 oct · taller</t>
+        </is>
+      </c>
+      <c r="D7" s="14" t="inlineStr">
+        <is>
           <t>Alado &amp; Co.</t>
         </is>
       </c>
-      <c r="D7" s="14" t="inlineStr">
-        <is>
-          <t>La tienda de Navidad</t>
-        </is>
-      </c>
       <c r="E7" s="14" t="inlineStr">
         <is>
+          <t>Recap del taller de cerámica</t>
+        </is>
+      </c>
+      <c r="F7" s="14" t="inlineStr">
+        <is>
           <t>Video</t>
         </is>
       </c>
-      <c r="F7" s="14" t="inlineStr">
-        <is>
-          <t>Núcleo</t>
-        </is>
-      </c>
       <c r="G7" s="14" t="inlineStr">
         <is>
+          <t>Núcleo</t>
+        </is>
+      </c>
+      <c r="H7" s="14" t="inlineStr">
+        <is>
           <t>A</t>
         </is>
       </c>
-      <c r="H7" s="7">
-        <f>IF(E7="Video",Presupuesto!$B$5,IF(E7="Carrusel",Presupuesto!$B$6,IF(E7="Historias",Presupuesto!$B$7,0)))</f>
+      <c r="I7" s="7">
+        <f>IF(F7="Video",Presupuesto!$B$5,IF(F7="Carrusel",Presupuesto!$B$6,IF(F7="Historias",Presupuesto!$B$7,0)))</f>
         <v/>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="12" t="inlineStr">
         <is>
-          <t>P07</t>
+          <t>07</t>
         </is>
       </c>
       <c r="B8" s="13" t="n">
-        <v>46322</v>
+        <v>46317</v>
       </c>
       <c r="C8" s="14" t="inlineStr">
         <is>
+          <t>lun 5 oct · atelier</t>
+        </is>
+      </c>
+      <c r="D8" s="14" t="inlineStr">
+        <is>
           <t>Bride</t>
         </is>
       </c>
-      <c r="D8" s="14" t="inlineStr">
-        <is>
-          <t>Oficio y detalle</t>
-        </is>
-      </c>
       <c r="E8" s="14" t="inlineStr">
         <is>
-          <t>Video</t>
+          <t>B10 · Único vs. alquilado</t>
         </is>
       </c>
       <c r="F8" s="14" t="inlineStr">
         <is>
-          <t>Núcleo</t>
+          <t>Carrusel</t>
         </is>
       </c>
       <c r="G8" s="14" t="inlineStr">
         <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="H8" s="7">
-        <f>IF(E8="Video",Presupuesto!$B$5,IF(E8="Carrusel",Presupuesto!$B$6,IF(E8="Historias",Presupuesto!$B$7,0)))</f>
+          <t>Núcleo</t>
+        </is>
+      </c>
+      <c r="H8" s="14" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="I8" s="7">
+        <f>IF(F8="Video",Presupuesto!$B$5,IF(F8="Carrusel",Presupuesto!$B$6,IF(F8="Historias",Presupuesto!$B$7,0)))</f>
         <v/>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="12" t="inlineStr">
         <is>
-          <t>P08</t>
+          <t>08</t>
         </is>
       </c>
       <c r="B9" s="13" t="n">
-        <v>46324</v>
+        <v>46319</v>
       </c>
       <c r="C9" s="14" t="inlineStr">
         <is>
+          <t>vie 23 oct · tienda</t>
+        </is>
+      </c>
+      <c r="D9" s="14" t="inlineStr">
+        <is>
           <t>Alado &amp; Co.</t>
         </is>
       </c>
-      <c r="D9" s="14" t="inlineStr">
-        <is>
-          <t>La casa se viste de Navidad</t>
-        </is>
-      </c>
       <c r="E9" s="14" t="inlineStr">
         <is>
+          <t>C5 · Recorrido por la tienda de Navidad</t>
+        </is>
+      </c>
+      <c r="F9" s="14" t="inlineStr">
+        <is>
           <t>Video</t>
         </is>
       </c>
-      <c r="F9" s="14" t="inlineStr">
-        <is>
-          <t>Núcleo</t>
-        </is>
-      </c>
       <c r="G9" s="14" t="inlineStr">
         <is>
+          <t>Núcleo</t>
+        </is>
+      </c>
+      <c r="H9" s="14" t="inlineStr">
+        <is>
           <t>A</t>
         </is>
       </c>
-      <c r="H9" s="7">
-        <f>IF(E9="Video",Presupuesto!$B$5,IF(E9="Carrusel",Presupuesto!$B$6,IF(E9="Historias",Presupuesto!$B$7,0)))</f>
+      <c r="I9" s="7">
+        <f>IF(F9="Video",Presupuesto!$B$5,IF(F9="Carrusel",Presupuesto!$B$6,IF(F9="Historias",Presupuesto!$B$7,0)))</f>
         <v/>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="12" t="inlineStr">
         <is>
-          <t>P09</t>
+          <t>09</t>
         </is>
       </c>
       <c r="B10" s="13" t="n">
-        <v>46329</v>
+        <v>46321</v>
       </c>
       <c r="C10" s="14" t="inlineStr">
         <is>
+          <t>vie 23 oct · tienda</t>
+        </is>
+      </c>
+      <c r="D10" s="14" t="inlineStr">
+        <is>
           <t>Alado &amp; Co.</t>
         </is>
       </c>
-      <c r="D10" s="14" t="inlineStr">
-        <is>
-          <t>Drop 1 · Flores (revelación)</t>
-        </is>
-      </c>
       <c r="E10" s="14" t="inlineStr">
         <is>
-          <t>Video</t>
+          <t>C20 · Cómo llegar a la tienda</t>
         </is>
       </c>
       <c r="F10" s="14" t="inlineStr">
         <is>
-          <t>Núcleo</t>
+          <t>Historias</t>
         </is>
       </c>
       <c r="G10" s="14" t="inlineStr">
         <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="H10" s="7">
-        <f>IF(E10="Video",Presupuesto!$B$5,IF(E10="Carrusel",Presupuesto!$B$6,IF(E10="Historias",Presupuesto!$B$7,0)))</f>
+          <t>Núcleo</t>
+        </is>
+      </c>
+      <c r="H10" s="14" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="I10" s="7">
+        <f>IF(F10="Video",Presupuesto!$B$5,IF(F10="Carrusel",Presupuesto!$B$6,IF(F10="Historias",Presupuesto!$B$7,0)))</f>
         <v/>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="12" t="inlineStr">
         <is>
-          <t>P10</t>
+          <t>10</t>
         </is>
       </c>
       <c r="B11" s="13" t="n">
-        <v>46331</v>
+        <v>46322</v>
       </c>
       <c r="C11" s="14" t="inlineStr">
         <is>
+          <t>sáb 17 oct · taller</t>
+        </is>
+      </c>
+      <c r="D11" s="14" t="inlineStr">
+        <is>
           <t>Alado &amp; Co.</t>
         </is>
       </c>
-      <c r="D11" s="14" t="inlineStr">
-        <is>
-          <t>Flores todo el año</t>
-        </is>
-      </c>
       <c r="E11" s="14" t="inlineStr">
         <is>
-          <t>Carrusel</t>
+          <t>C1 · Cómo se pinta una pieza (1)</t>
         </is>
       </c>
       <c r="F11" s="14" t="inlineStr">
         <is>
-          <t>Núcleo</t>
+          <t>Video</t>
         </is>
       </c>
       <c r="G11" s="14" t="inlineStr">
         <is>
+          <t>Núcleo</t>
+        </is>
+      </c>
+      <c r="H11" s="14" t="inlineStr">
+        <is>
           <t>B</t>
         </is>
       </c>
-      <c r="H11" s="7">
-        <f>IF(E11="Video",Presupuesto!$B$5,IF(E11="Carrusel",Presupuesto!$B$6,IF(E11="Historias",Presupuesto!$B$7,0)))</f>
+      <c r="I11" s="7">
+        <f>IF(F11="Video",Presupuesto!$B$5,IF(F11="Carrusel",Presupuesto!$B$6,IF(F11="Historias",Presupuesto!$B$7,0)))</f>
         <v/>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="12" t="inlineStr">
         <is>
-          <t>P11</t>
+          <t>11</t>
         </is>
       </c>
       <c r="B12" s="13" t="n">
-        <v>46336</v>
+        <v>46324</v>
       </c>
       <c r="C12" s="14" t="inlineStr">
         <is>
+          <t>vie 16 oct · casa de Andrés</t>
+        </is>
+      </c>
+      <c r="D12" s="14" t="inlineStr">
+        <is>
           <t>Alado &amp; Co.</t>
         </is>
       </c>
-      <c r="D12" s="14" t="inlineStr">
-        <is>
-          <t>Drop 2 · Caballos a cuadros (revelación)</t>
-        </is>
-      </c>
       <c r="E12" s="14" t="inlineStr">
         <is>
+          <t>La casa se viste de Navidad</t>
+        </is>
+      </c>
+      <c r="F12" s="14" t="inlineStr">
+        <is>
           <t>Video</t>
         </is>
       </c>
-      <c r="F12" s="14" t="inlineStr">
-        <is>
-          <t>Núcleo</t>
-        </is>
-      </c>
       <c r="G12" s="14" t="inlineStr">
         <is>
+          <t>Núcleo</t>
+        </is>
+      </c>
+      <c r="H12" s="14" t="inlineStr">
+        <is>
           <t>A</t>
         </is>
       </c>
-      <c r="H12" s="7">
-        <f>IF(E12="Video",Presupuesto!$B$5,IF(E12="Carrusel",Presupuesto!$B$6,IF(E12="Historias",Presupuesto!$B$7,0)))</f>
+      <c r="I12" s="7">
+        <f>IF(F12="Video",Presupuesto!$B$5,IF(F12="Carrusel",Presupuesto!$B$6,IF(F12="Historias",Presupuesto!$B$7,0)))</f>
         <v/>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="12" t="inlineStr">
         <is>
-          <t>P12</t>
+          <t>12</t>
         </is>
       </c>
       <c r="B13" s="13" t="n">
-        <v>46338</v>
+        <v>46328</v>
       </c>
       <c r="C13" s="14" t="inlineStr">
         <is>
-          <t>Bride</t>
+          <t>vie 23 oct · tienda</t>
         </is>
       </c>
       <c r="D13" s="14" t="inlineStr">
         <is>
-          <t>El figurín enmarcado</t>
+          <t>Alado &amp; Co.</t>
         </is>
       </c>
       <c r="E13" s="14" t="inlineStr">
         <is>
-          <t>Video</t>
+          <t>C19 · Esta semana en la tienda (1)</t>
         </is>
       </c>
       <c r="F13" s="14" t="inlineStr">
         <is>
-          <t>Núcleo</t>
+          <t>Historias</t>
         </is>
       </c>
       <c r="G13" s="14" t="inlineStr">
         <is>
+          <t>Núcleo</t>
+        </is>
+      </c>
+      <c r="H13" s="14" t="inlineStr">
+        <is>
           <t>B</t>
         </is>
       </c>
-      <c r="H13" s="7">
-        <f>IF(E13="Video",Presupuesto!$B$5,IF(E13="Carrusel",Presupuesto!$B$6,IF(E13="Historias",Presupuesto!$B$7,0)))</f>
+      <c r="I13" s="7">
+        <f>IF(F13="Video",Presupuesto!$B$5,IF(F13="Carrusel",Presupuesto!$B$6,IF(F13="Historias",Presupuesto!$B$7,0)))</f>
         <v/>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="12" t="inlineStr">
         <is>
-          <t>P13</t>
+          <t>13</t>
         </is>
       </c>
       <c r="B14" s="13" t="n">
-        <v>46343</v>
+        <v>46329</v>
       </c>
       <c r="C14" s="14" t="inlineStr">
         <is>
+          <t>vie 16 oct · casa de Andrés</t>
+        </is>
+      </c>
+      <c r="D14" s="14" t="inlineStr">
+        <is>
           <t>Alado &amp; Co.</t>
         </is>
       </c>
-      <c r="D14" s="14" t="inlineStr">
-        <is>
-          <t>Drop 3 · Ángeles y ciervos (revelación)</t>
-        </is>
-      </c>
       <c r="E14" s="14" t="inlineStr">
         <is>
+          <t>Drop 1 · Flores</t>
+        </is>
+      </c>
+      <c r="F14" s="14" t="inlineStr">
+        <is>
           <t>Video</t>
         </is>
       </c>
-      <c r="F14" s="14" t="inlineStr">
-        <is>
-          <t>Núcleo</t>
-        </is>
-      </c>
       <c r="G14" s="14" t="inlineStr">
         <is>
+          <t>Núcleo</t>
+        </is>
+      </c>
+      <c r="H14" s="14" t="inlineStr">
+        <is>
           <t>A</t>
         </is>
       </c>
-      <c r="H14" s="7">
-        <f>IF(E14="Video",Presupuesto!$B$5,IF(E14="Carrusel",Presupuesto!$B$6,IF(E14="Historias",Presupuesto!$B$7,0)))</f>
+      <c r="I14" s="7">
+        <f>IF(F14="Video",Presupuesto!$B$5,IF(F14="Carrusel",Presupuesto!$B$6,IF(F14="Historias",Presupuesto!$B$7,0)))</f>
         <v/>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="12" t="inlineStr">
         <is>
-          <t>P14</t>
+          <t>14</t>
         </is>
       </c>
       <c r="B15" s="13" t="n">
-        <v>46345</v>
+        <v>46331</v>
       </c>
       <c r="C15" s="14" t="inlineStr">
         <is>
-          <t>Celebration</t>
+          <t>mar 3 nov · casa o tienda</t>
         </is>
       </c>
       <c r="D15" s="14" t="inlineStr">
         <is>
-          <t>Prom y 15s: tu vestido, único</t>
+          <t>Alado &amp; Co.</t>
         </is>
       </c>
       <c r="E15" s="14" t="inlineStr">
         <is>
-          <t>Carrusel</t>
+          <t>C10 · Pon la mesa con tus piezas pintadas</t>
         </is>
       </c>
       <c r="F15" s="14" t="inlineStr">
         <is>
-          <t>Núcleo</t>
+          <t>Video</t>
         </is>
       </c>
       <c r="G15" s="14" t="inlineStr">
         <is>
+          <t>Núcleo</t>
+        </is>
+      </c>
+      <c r="H15" s="14" t="inlineStr">
+        <is>
           <t>B</t>
         </is>
       </c>
-      <c r="H15" s="7">
-        <f>IF(E15="Video",Presupuesto!$B$5,IF(E15="Carrusel",Presupuesto!$B$6,IF(E15="Historias",Presupuesto!$B$7,0)))</f>
+      <c r="I15" s="7">
+        <f>IF(F15="Video",Presupuesto!$B$5,IF(F15="Carrusel",Presupuesto!$B$6,IF(F15="Historias",Presupuesto!$B$7,0)))</f>
         <v/>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="12" t="inlineStr">
         <is>
-          <t>P15</t>
+          <t>15</t>
         </is>
       </c>
       <c r="B16" s="13" t="n">
-        <v>46350</v>
+        <v>46333</v>
       </c>
       <c r="C16" s="14" t="inlineStr">
         <is>
-          <t>Bride</t>
+          <t>vie 16 oct · casa de Andrés</t>
         </is>
       </c>
       <c r="D16" s="14" t="inlineStr">
         <is>
-          <t>Notas de Alejo: qué se va y qué se queda</t>
+          <t>Alado &amp; Co.</t>
         </is>
       </c>
       <c r="E16" s="14" t="inlineStr">
         <is>
-          <t>Video</t>
+          <t>C11 · Cómo vestir una mesa por capas</t>
         </is>
       </c>
       <c r="F16" s="14" t="inlineStr">
         <is>
-          <t>Núcleo</t>
+          <t>Carrusel</t>
         </is>
       </c>
       <c r="G16" s="14" t="inlineStr">
         <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="H16" s="7">
-        <f>IF(E16="Video",Presupuesto!$B$5,IF(E16="Carrusel",Presupuesto!$B$6,IF(E16="Historias",Presupuesto!$B$7,0)))</f>
+          <t>Núcleo</t>
+        </is>
+      </c>
+      <c r="H16" s="14" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="I16" s="7">
+        <f>IF(F16="Video",Presupuesto!$B$5,IF(F16="Carrusel",Presupuesto!$B$6,IF(F16="Historias",Presupuesto!$B$7,0)))</f>
         <v/>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="12" t="inlineStr">
         <is>
-          <t>P16</t>
+          <t>16</t>
         </is>
       </c>
       <c r="B17" s="13" t="n">
-        <v>46352</v>
+        <v>46336</v>
       </c>
       <c r="C17" s="14" t="inlineStr">
         <is>
-          <t>Alado</t>
+          <t>vie 16 oct · casa de Andrés</t>
         </is>
       </c>
       <c r="D17" s="14" t="inlineStr">
         <is>
-          <t>Regala Alado (guía de regalos)</t>
+          <t>Alado &amp; Co.</t>
         </is>
       </c>
       <c r="E17" s="14" t="inlineStr">
         <is>
-          <t>Carrusel</t>
+          <t>Drop 2 · Caballos a cuadros</t>
         </is>
       </c>
       <c r="F17" s="14" t="inlineStr">
         <is>
-          <t>Núcleo</t>
+          <t>Video</t>
         </is>
       </c>
       <c r="G17" s="14" t="inlineStr">
         <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="H17" s="7">
-        <f>IF(E17="Video",Presupuesto!$B$5,IF(E17="Carrusel",Presupuesto!$B$6,IF(E17="Historias",Presupuesto!$B$7,0)))</f>
+          <t>Núcleo</t>
+        </is>
+      </c>
+      <c r="H17" s="14" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="I17" s="7">
+        <f>IF(F17="Video",Presupuesto!$B$5,IF(F17="Carrusel",Presupuesto!$B$6,IF(F17="Historias",Presupuesto!$B$7,0)))</f>
         <v/>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="12" t="inlineStr">
         <is>
-          <t>P17</t>
+          <t>17</t>
         </is>
       </c>
       <c r="B18" s="13" t="n">
-        <v>46357</v>
+        <v>46338</v>
       </c>
       <c r="C18" s="14" t="inlineStr">
         <is>
+          <t>lun 5 oct · atelier</t>
+        </is>
+      </c>
+      <c r="D18" s="14" t="inlineStr">
+        <is>
           <t>Bride</t>
         </is>
       </c>
-      <c r="D18" s="14" t="inlineStr">
-        <is>
-          <t>Agenda tu cita antes de vacaciones</t>
-        </is>
-      </c>
       <c r="E18" s="14" t="inlineStr">
         <is>
+          <t>B11 · Del primer lápiz a la entrega</t>
+        </is>
+      </c>
+      <c r="F18" s="14" t="inlineStr">
+        <is>
           <t>Carrusel</t>
         </is>
       </c>
-      <c r="F18" s="14" t="inlineStr">
-        <is>
-          <t>Núcleo</t>
-        </is>
-      </c>
       <c r="G18" s="14" t="inlineStr">
         <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="H18" s="7">
-        <f>IF(E18="Video",Presupuesto!$B$5,IF(E18="Carrusel",Presupuesto!$B$6,IF(E18="Historias",Presupuesto!$B$7,0)))</f>
+          <t>Núcleo</t>
+        </is>
+      </c>
+      <c r="H18" s="14" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="I18" s="7">
+        <f>IF(F18="Video",Presupuesto!$B$5,IF(F18="Carrusel",Presupuesto!$B$6,IF(F18="Historias",Presupuesto!$B$7,0)))</f>
         <v/>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="12" t="inlineStr">
         <is>
-          <t>H1</t>
+          <t>18</t>
         </is>
       </c>
       <c r="B19" s="13" t="n">
-        <v>46300</v>
+        <v>46342</v>
       </c>
       <c r="C19" s="14" t="inlineStr">
         <is>
-          <t>Bride</t>
+          <t>vie 6 nov · tienda</t>
         </is>
       </c>
       <c r="D19" s="14" t="inlineStr">
         <is>
-          <t>Destacado fijo «Bride» (montaje único)</t>
+          <t>Alado &amp; Co.</t>
         </is>
       </c>
       <c r="E19" s="14" t="inlineStr">
         <is>
+          <t>C19 · Esta semana en la tienda (2)</t>
+        </is>
+      </c>
+      <c r="F19" s="14" t="inlineStr">
+        <is>
           <t>Historias</t>
         </is>
       </c>
-      <c r="F19" s="14" t="inlineStr">
-        <is>
-          <t>Historias (opcional)</t>
-        </is>
-      </c>
       <c r="G19" s="14" t="inlineStr">
         <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="H19" s="7">
-        <f>IF(E19="Video",Presupuesto!$B$5,IF(E19="Carrusel",Presupuesto!$B$6,IF(E19="Historias",Presupuesto!$B$7,0)))</f>
+          <t>Núcleo</t>
+        </is>
+      </c>
+      <c r="H19" s="14" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="I19" s="7">
+        <f>IF(F19="Video",Presupuesto!$B$5,IF(F19="Carrusel",Presupuesto!$B$6,IF(F19="Historias",Presupuesto!$B$7,0)))</f>
         <v/>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="12" t="inlineStr">
         <is>
-          <t>H2</t>
+          <t>19</t>
         </is>
       </c>
       <c r="B20" s="13" t="n">
-        <v>46312</v>
+        <v>46343</v>
       </c>
       <c r="C20" s="14" t="inlineStr">
         <is>
+          <t>vie 16 oct · casa de Andrés</t>
+        </is>
+      </c>
+      <c r="D20" s="14" t="inlineStr">
+        <is>
           <t>Alado &amp; Co.</t>
         </is>
       </c>
-      <c r="D20" s="14" t="inlineStr">
-        <is>
-          <t>Taller de cerámica en vivo</t>
-        </is>
-      </c>
       <c r="E20" s="14" t="inlineStr">
         <is>
-          <t>Historias</t>
+          <t>Drop 3 · Ángeles y ciervos</t>
         </is>
       </c>
       <c r="F20" s="14" t="inlineStr">
         <is>
-          <t>Historias (opcional)</t>
+          <t>Video</t>
         </is>
       </c>
       <c r="G20" s="14" t="inlineStr">
         <is>
+          <t>Núcleo</t>
+        </is>
+      </c>
+      <c r="H20" s="14" t="inlineStr">
+        <is>
           <t>A</t>
         </is>
       </c>
-      <c r="H20" s="7">
-        <f>IF(E20="Video",Presupuesto!$B$5,IF(E20="Carrusel",Presupuesto!$B$6,IF(E20="Historias",Presupuesto!$B$7,0)))</f>
+      <c r="I20" s="7">
+        <f>IF(F20="Video",Presupuesto!$B$5,IF(F20="Carrusel",Presupuesto!$B$6,IF(F20="Historias",Presupuesto!$B$7,0)))</f>
         <v/>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="12" t="inlineStr">
         <is>
-          <t>H3</t>
+          <t>20</t>
         </is>
       </c>
       <c r="B21" s="13" t="n">
-        <v>46328</v>
+        <v>46345</v>
       </c>
       <c r="C21" s="14" t="inlineStr">
         <is>
-          <t>Alado &amp; Co.</t>
+          <t>lun 5 oct · atelier</t>
         </is>
       </c>
       <c r="D21" s="14" t="inlineStr">
         <is>
-          <t>Semana de lanzamiento de los drops</t>
+          <t>Celebration</t>
         </is>
       </c>
       <c r="E21" s="14" t="inlineStr">
         <is>
-          <t>Historias</t>
+          <t>B15 · Prom y 15s: tu vestido, único</t>
         </is>
       </c>
       <c r="F21" s="14" t="inlineStr">
         <is>
-          <t>Historias (opcional)</t>
+          <t>Carrusel</t>
         </is>
       </c>
       <c r="G21" s="14" t="inlineStr">
         <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="H21" s="7">
-        <f>IF(E21="Video",Presupuesto!$B$5,IF(E21="Carrusel",Presupuesto!$B$6,IF(E21="Historias",Presupuesto!$B$7,0)))</f>
+          <t>Núcleo</t>
+        </is>
+      </c>
+      <c r="H21" s="14" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="I21" s="7">
+        <f>IF(F21="Video",Presupuesto!$B$5,IF(F21="Carrusel",Presupuesto!$B$6,IF(F21="Historias",Presupuesto!$B$7,0)))</f>
         <v/>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="12" t="inlineStr">
         <is>
-          <t>H4</t>
+          <t>21</t>
         </is>
       </c>
       <c r="B22" s="13" t="n">
-        <v>46356</v>
+        <v>46347</v>
       </c>
       <c r="C22" s="14" t="inlineStr">
         <is>
-          <t>Bride</t>
+          <t>jue 12 nov · casa de Andrés</t>
         </is>
       </c>
       <c r="D22" s="14" t="inlineStr">
         <is>
-          <t>Última llamada antes de vacaciones</t>
+          <t>Alado &amp; Co.</t>
         </is>
       </c>
       <c r="E22" s="14" t="inlineStr">
         <is>
-          <t>Historias</t>
+          <t>Receta de Navidad en la mesa Alado</t>
         </is>
       </c>
       <c r="F22" s="14" t="inlineStr">
         <is>
-          <t>Historias (opcional)</t>
+          <t>Video</t>
         </is>
       </c>
       <c r="G22" s="14" t="inlineStr">
         <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="H22" s="7">
-        <f>IF(E22="Video",Presupuesto!$B$5,IF(E22="Carrusel",Presupuesto!$B$6,IF(E22="Historias",Presupuesto!$B$7,0)))</f>
+          <t>Núcleo</t>
+        </is>
+      </c>
+      <c r="H22" s="14" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="I22" s="7">
+        <f>IF(F22="Video",Presupuesto!$B$5,IF(F22="Carrusel",Presupuesto!$B$6,IF(F22="Historias",Presupuesto!$B$7,0)))</f>
         <v/>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="12" t="inlineStr">
         <is>
-          <t>B1</t>
+          <t>22</t>
         </is>
       </c>
       <c r="B23" s="13" t="n">
-        <v>46371</v>
+        <v>46349</v>
       </c>
       <c r="C23" s="14" t="inlineStr">
         <is>
-          <t>Alado &amp; Co.</t>
+          <t>mar 17 nov · Alejo</t>
         </is>
       </c>
       <c r="D23" s="14" t="inlineStr">
         <is>
-          <t>No es solo Navidad (flores y caballos todo el año)</t>
+          <t>Bride</t>
         </is>
       </c>
       <c r="E23" s="14" t="inlineStr">
         <is>
-          <t>Video</t>
+          <t>B17 · Caja de preguntas con Alejo</t>
         </is>
       </c>
       <c r="F23" s="14" t="inlineStr">
         <is>
-          <t>Fase B</t>
+          <t>Historias</t>
         </is>
       </c>
       <c r="G23" s="14" t="inlineStr">
         <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="H23" s="7">
-        <f>IF(E23="Video",Presupuesto!$B$5,IF(E23="Carrusel",Presupuesto!$B$6,IF(E23="Historias",Presupuesto!$B$7,0)))</f>
+          <t>Núcleo</t>
+        </is>
+      </c>
+      <c r="H23" s="14" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="I23" s="7">
+        <f>IF(F23="Video",Presupuesto!$B$5,IF(F23="Carrusel",Presupuesto!$B$6,IF(F23="Historias",Presupuesto!$B$7,0)))</f>
         <v/>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="12" t="inlineStr">
         <is>
-          <t>B2</t>
+          <t>23</t>
         </is>
       </c>
       <c r="B24" s="13" t="n">
-        <v>46374</v>
+        <v>46350</v>
       </c>
       <c r="C24" s="14" t="inlineStr">
         <is>
-          <t>Alado</t>
+          <t>mar 17 nov · Alejo</t>
         </is>
       </c>
       <c r="D24" s="14" t="inlineStr">
         <is>
-          <t>Regala Alado (envolver, ASMR)</t>
+          <t>Bride</t>
         </is>
       </c>
       <c r="E24" s="14" t="inlineStr">
         <is>
+          <t>B3 · Notas de Alejo (manuscritas)</t>
+        </is>
+      </c>
+      <c r="F24" s="14" t="inlineStr">
+        <is>
           <t>Video</t>
         </is>
       </c>
-      <c r="F24" s="14" t="inlineStr">
-        <is>
-          <t>Fase B</t>
-        </is>
-      </c>
       <c r="G24" s="14" t="inlineStr">
         <is>
+          <t>Núcleo</t>
+        </is>
+      </c>
+      <c r="H24" s="14" t="inlineStr">
+        <is>
           <t>A</t>
         </is>
       </c>
-      <c r="H24" s="7">
-        <f>IF(E24="Video",Presupuesto!$B$5,IF(E24="Carrusel",Presupuesto!$B$6,IF(E24="Historias",Presupuesto!$B$7,0)))</f>
+      <c r="I24" s="7">
+        <f>IF(F24="Video",Presupuesto!$B$5,IF(F24="Carrusel",Presupuesto!$B$6,IF(F24="Historias",Presupuesto!$B$7,0)))</f>
         <v/>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="12" t="inlineStr">
         <is>
-          <t>B3</t>
+          <t>24</t>
         </is>
       </c>
       <c r="B25" s="13" t="n">
-        <v>46378</v>
+        <v>46352</v>
       </c>
       <c r="C25" s="14" t="inlineStr">
         <is>
+          <t>jue 19 nov · tienda</t>
+        </is>
+      </c>
+      <c r="D25" s="14" t="inlineStr">
+        <is>
           <t>Alado &amp; Co.</t>
         </is>
       </c>
-      <c r="D25" s="14" t="inlineStr">
-        <is>
-          <t>Cómo montar una mesa que se recuerde</t>
-        </is>
-      </c>
       <c r="E25" s="14" t="inlineStr">
         <is>
+          <t>Armamos una ancheta Alado</t>
+        </is>
+      </c>
+      <c r="F25" s="14" t="inlineStr">
+        <is>
           <t>Video</t>
         </is>
       </c>
-      <c r="F25" s="14" t="inlineStr">
-        <is>
-          <t>Fase B</t>
-        </is>
-      </c>
       <c r="G25" s="14" t="inlineStr">
         <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="H25" s="7">
-        <f>IF(E25="Video",Presupuesto!$B$5,IF(E25="Carrusel",Presupuesto!$B$6,IF(E25="Historias",Presupuesto!$B$7,0)))</f>
+          <t>Núcleo</t>
+        </is>
+      </c>
+      <c r="H25" s="14" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="I25" s="7">
+        <f>IF(F25="Video",Presupuesto!$B$5,IF(F25="Carrusel",Presupuesto!$B$6,IF(F25="Historias",Presupuesto!$B$7,0)))</f>
         <v/>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="12" t="inlineStr">
         <is>
-          <t>B4</t>
+          <t>25</t>
         </is>
       </c>
       <c r="B26" s="13" t="n">
-        <v>46385</v>
+        <v>46354</v>
       </c>
       <c r="C26" s="14" t="inlineStr">
         <is>
+          <t>sáb 21 nov · El Retiro</t>
+        </is>
+      </c>
+      <c r="D26" s="14" t="inlineStr">
+        <is>
           <t>Alado &amp; Co.</t>
         </is>
       </c>
-      <c r="D26" s="14" t="inlineStr">
-        <is>
-          <t>Del dibujo al textil</t>
-        </is>
-      </c>
       <c r="E26" s="14" t="inlineStr">
         <is>
-          <t>Video</t>
+          <t>C14 · Un día en El Retiro en Navidad</t>
         </is>
       </c>
       <c r="F26" s="14" t="inlineStr">
         <is>
-          <t>Fase B</t>
+          <t>Carrusel</t>
         </is>
       </c>
       <c r="G26" s="14" t="inlineStr">
         <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="H26" s="7">
-        <f>IF(E26="Video",Presupuesto!$B$5,IF(E26="Carrusel",Presupuesto!$B$6,IF(E26="Historias",Presupuesto!$B$7,0)))</f>
+          <t>Núcleo</t>
+        </is>
+      </c>
+      <c r="H26" s="14" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="I26" s="7">
+        <f>IF(F26="Video",Presupuesto!$B$5,IF(F26="Carrusel",Presupuesto!$B$6,IF(F26="Historias",Presupuesto!$B$7,0)))</f>
         <v/>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="12" t="inlineStr">
         <is>
-          <t>B5</t>
+          <t>26</t>
         </is>
       </c>
       <c r="B27" s="13" t="n">
-        <v>46392</v>
+        <v>46356</v>
       </c>
       <c r="C27" s="14" t="inlineStr">
         <is>
+          <t>mar 17 nov · Alejo</t>
+        </is>
+      </c>
+      <c r="D27" s="14" t="inlineStr">
+        <is>
           <t>Bride</t>
         </is>
       </c>
-      <c r="D27" s="14" t="inlineStr">
-        <is>
-          <t>Notas de Alejo: novias 2027</t>
-        </is>
-      </c>
       <c r="E27" s="14" t="inlineStr">
         <is>
-          <t>Carrusel</t>
+          <t>B20 · Agenda abierta hasta el 11 de diciembre</t>
         </is>
       </c>
       <c r="F27" s="14" t="inlineStr">
         <is>
-          <t>Fase B</t>
+          <t>Historias</t>
         </is>
       </c>
       <c r="G27" s="14" t="inlineStr">
         <is>
+          <t>Núcleo</t>
+        </is>
+      </c>
+      <c r="H27" s="14" t="inlineStr">
+        <is>
           <t>A</t>
         </is>
       </c>
-      <c r="H27" s="7">
-        <f>IF(E27="Video",Presupuesto!$B$5,IF(E27="Carrusel",Presupuesto!$B$6,IF(E27="Historias",Presupuesto!$B$7,0)))</f>
+      <c r="I27" s="7">
+        <f>IF(F27="Video",Presupuesto!$B$5,IF(F27="Carrusel",Presupuesto!$B$6,IF(F27="Historias",Presupuesto!$B$7,0)))</f>
         <v/>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="12" t="inlineStr">
         <is>
-          <t>B6</t>
+          <t>V1</t>
         </is>
       </c>
       <c r="B28" s="13" t="n">
+        <v>46371</v>
+      </c>
+      <c r="C28" s="14" t="inlineStr">
+        <is>
+          <t>1–9 dic · banco</t>
+        </is>
+      </c>
+      <c r="D28" s="14" t="inlineStr">
+        <is>
+          <t>Alado &amp; Co.</t>
+        </is>
+      </c>
+      <c r="E28" s="14" t="inlineStr">
+        <is>
+          <t>No es solo Navidad (flores y caballos todo el año)</t>
+        </is>
+      </c>
+      <c r="F28" s="14" t="inlineStr">
+        <is>
+          <t>Video</t>
+        </is>
+      </c>
+      <c r="G28" s="14" t="inlineStr">
+        <is>
+          <t>Fase B</t>
+        </is>
+      </c>
+      <c r="H28" s="14" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="I28" s="7">
+        <f>IF(F28="Video",Presupuesto!$B$5,IF(F28="Carrusel",Presupuesto!$B$6,IF(F28="Historias",Presupuesto!$B$7,0)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="12" t="inlineStr">
+        <is>
+          <t>V2</t>
+        </is>
+      </c>
+      <c r="B29" s="13" t="n">
+        <v>46374</v>
+      </c>
+      <c r="C29" s="14" t="inlineStr">
+        <is>
+          <t>1–9 dic · banco</t>
+        </is>
+      </c>
+      <c r="D29" s="14" t="inlineStr">
+        <is>
+          <t>Alado</t>
+        </is>
+      </c>
+      <c r="E29" s="14" t="inlineStr">
+        <is>
+          <t>Regala Alado (envolver)</t>
+        </is>
+      </c>
+      <c r="F29" s="14" t="inlineStr">
+        <is>
+          <t>Video</t>
+        </is>
+      </c>
+      <c r="G29" s="14" t="inlineStr">
+        <is>
+          <t>Fase B</t>
+        </is>
+      </c>
+      <c r="H29" s="14" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="I29" s="7">
+        <f>IF(F29="Video",Presupuesto!$B$5,IF(F29="Carrusel",Presupuesto!$B$6,IF(F29="Historias",Presupuesto!$B$7,0)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="12" t="inlineStr">
+        <is>
+          <t>V3</t>
+        </is>
+      </c>
+      <c r="B30" s="13" t="n">
+        <v>46378</v>
+      </c>
+      <c r="C30" s="14" t="inlineStr">
+        <is>
+          <t>1–9 dic · banco</t>
+        </is>
+      </c>
+      <c r="D30" s="14" t="inlineStr">
+        <is>
+          <t>Alado &amp; Co.</t>
+        </is>
+      </c>
+      <c r="E30" s="14" t="inlineStr">
+        <is>
+          <t>Cómo montar una mesa que se recuerde</t>
+        </is>
+      </c>
+      <c r="F30" s="14" t="inlineStr">
+        <is>
+          <t>Video</t>
+        </is>
+      </c>
+      <c r="G30" s="14" t="inlineStr">
+        <is>
+          <t>Fase B</t>
+        </is>
+      </c>
+      <c r="H30" s="14" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="I30" s="7">
+        <f>IF(F30="Video",Presupuesto!$B$5,IF(F30="Carrusel",Presupuesto!$B$6,IF(F30="Historias",Presupuesto!$B$7,0)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="12" t="inlineStr">
+        <is>
+          <t>V4</t>
+        </is>
+      </c>
+      <c r="B31" s="13" t="n">
+        <v>46385</v>
+      </c>
+      <c r="C31" s="14" t="inlineStr">
+        <is>
+          <t>1–9 dic · banco</t>
+        </is>
+      </c>
+      <c r="D31" s="14" t="inlineStr">
+        <is>
+          <t>Alado &amp; Co.</t>
+        </is>
+      </c>
+      <c r="E31" s="14" t="inlineStr">
+        <is>
+          <t>C1 · Cómo se pinta una pieza (2)</t>
+        </is>
+      </c>
+      <c r="F31" s="14" t="inlineStr">
+        <is>
+          <t>Video</t>
+        </is>
+      </c>
+      <c r="G31" s="14" t="inlineStr">
+        <is>
+          <t>Fase B</t>
+        </is>
+      </c>
+      <c r="H31" s="14" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="I31" s="7">
+        <f>IF(F31="Video",Presupuesto!$B$5,IF(F31="Carrusel",Presupuesto!$B$6,IF(F31="Historias",Presupuesto!$B$7,0)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="12" t="inlineStr">
+        <is>
+          <t>V5</t>
+        </is>
+      </c>
+      <c r="B32" s="13" t="n">
+        <v>46392</v>
+      </c>
+      <c r="C32" s="14" t="inlineStr">
+        <is>
+          <t>1–9 dic · banco</t>
+        </is>
+      </c>
+      <c r="D32" s="14" t="inlineStr">
+        <is>
+          <t>Bride</t>
+        </is>
+      </c>
+      <c r="E32" s="14" t="inlineStr">
+        <is>
+          <t>Notas de Alejo: novias 2027</t>
+        </is>
+      </c>
+      <c r="F32" s="14" t="inlineStr">
+        <is>
+          <t>Carrusel</t>
+        </is>
+      </c>
+      <c r="G32" s="14" t="inlineStr">
+        <is>
+          <t>Fase B</t>
+        </is>
+      </c>
+      <c r="H32" s="14" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="I32" s="7">
+        <f>IF(F32="Video",Presupuesto!$B$5,IF(F32="Carrusel",Presupuesto!$B$6,IF(F32="Historias",Presupuesto!$B$7,0)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="12" t="inlineStr">
+        <is>
+          <t>V6</t>
+        </is>
+      </c>
+      <c r="B33" s="13" t="n">
         <v>46396</v>
       </c>
-      <c r="C28" s="14" t="inlineStr">
+      <c r="C33" s="14" t="inlineStr">
+        <is>
+          <t>1–9 dic · banco</t>
+        </is>
+      </c>
+      <c r="D33" s="14" t="inlineStr">
         <is>
           <t>Bride</t>
         </is>
       </c>
-      <c r="D28" s="14" t="inlineStr">
+      <c r="E33" s="14" t="inlineStr">
         <is>
           <t>Cómo agendar tu cita desde el 12 de enero</t>
         </is>
       </c>
-      <c r="E28" s="14" t="inlineStr">
+      <c r="F33" s="14" t="inlineStr">
         <is>
           <t>Carrusel</t>
         </is>
       </c>
-      <c r="F28" s="14" t="inlineStr">
+      <c r="G33" s="14" t="inlineStr">
         <is>
           <t>Fase B</t>
         </is>
       </c>
-      <c r="G28" s="14" t="inlineStr">
+      <c r="H33" s="14" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
-      <c r="H28" s="7">
-        <f>IF(E28="Video",Presupuesto!$B$5,IF(E28="Carrusel",Presupuesto!$B$6,IF(E28="Historias",Presupuesto!$B$7,0)))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="30">
-      <c r="D30" s="2" t="inlineStr">
-        <is>
-          <t>Puedes cambiar fecha, formato, fase o prioridad; el presupuesto se recalcula solo.</t>
+      <c r="I33" s="7">
+        <f>IF(F33="Video",Presupuesto!$B$5,IF(F33="Carrusel",Presupuesto!$B$6,IF(F33="Historias",Presupuesto!$B$7,0)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="35">
+      <c r="E35" s="2" t="inlineStr">
+        <is>
+          <t>Cambia fecha, formato, fase o prioridad y el presupuesto se recalcula solo.</t>
         </is>
       </c>
     </row>
   </sheetData>
   <dataValidations count="3">
-    <dataValidation sqref="E2:E48" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="F2:F53" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Video,Carrusel,Historias"</formula1>
     </dataValidation>
-    <dataValidation sqref="F2:F48" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"Núcleo,Historias (opcional),Fase B"</formula1>
+    <dataValidation sqref="G2:G53" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Núcleo,Fase B"</formula1>
     </dataValidation>
-    <dataValidation sqref="G2:G48" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="H2:H53" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"A,B"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Update rates to reel 200k, carousel 170k, story set 120k; recalc budget, plan and data
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FV7y6XEE3x9ogCMyfe3pnd
</commit_message>
<xml_diff>
--- a/docs/sesion-2026-10-02/presupuesto-contenido-oct-dic.xlsx
+++ b/docs/sesion-2026-10-02/presupuesto-contenido-oct-dic.xlsx
@@ -530,7 +530,7 @@
         </is>
       </c>
       <c r="B5" s="5" t="n">
-        <v>210000</v>
+        <v>200000</v>
       </c>
     </row>
     <row r="6">
@@ -540,7 +540,7 @@
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>150000</v>
+        <v>170000</v>
       </c>
     </row>
     <row r="7">
@@ -550,7 +550,7 @@
         </is>
       </c>
       <c r="B7" s="5" t="n">
-        <v>180000</v>
+        <v>120000</v>
       </c>
     </row>
     <row r="9">

</xml_diff>

<commit_message>
Reduce ceramics workshop content to 4 pieces; recalc plan to 4.18M and update deck data
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FV7y6XEE3x9ogCMyfe3pnd
</commit_message>
<xml_diff>
--- a/docs/sesion-2026-10-02/presupuesto-contenido-oct-dic.xlsx
+++ b/docs/sesion-2026-10-02/presupuesto-contenido-oct-dic.xlsx
@@ -567,7 +567,7 @@
         </is>
       </c>
       <c r="B10" s="6">
-        <f>COUNTIFS(Calendario!$F$2:$F$53,"Video",Calendario!$G$2:$G$53,"Núcleo")</f>
+        <f>COUNTIFS(Calendario!$F$2:$F$52,"Video",Calendario!$G$2:$G$52,"Núcleo")</f>
         <v/>
       </c>
     </row>
@@ -578,7 +578,7 @@
         </is>
       </c>
       <c r="B11" s="6">
-        <f>COUNTIFS(Calendario!$F$2:$F$53,"Carrusel",Calendario!$G$2:$G$53,"Núcleo")</f>
+        <f>COUNTIFS(Calendario!$F$2:$F$52,"Carrusel",Calendario!$G$2:$G$52,"Núcleo")</f>
         <v/>
       </c>
     </row>
@@ -589,7 +589,7 @@
         </is>
       </c>
       <c r="B12" s="6">
-        <f>COUNTIFS(Calendario!$F$2:$F$53,"Historias",Calendario!$G$2:$G$53,"Núcleo")</f>
+        <f>COUNTIFS(Calendario!$F$2:$F$52,"Historias",Calendario!$G$2:$G$52,"Núcleo")</f>
         <v/>
       </c>
     </row>
@@ -600,7 +600,7 @@
         </is>
       </c>
       <c r="B13" s="6">
-        <f>COUNTIFS(Calendario!$G$2:$G$53,"Fase B")</f>
+        <f>COUNTIFS(Calendario!$G$2:$G$52,"Fase B")</f>
         <v/>
       </c>
     </row>
@@ -618,7 +618,7 @@
         </is>
       </c>
       <c r="B16" s="7">
-        <f>SUMIFS(Calendario!$I$2:$I$53,Calendario!$G$2:$G$53,"Núcleo",Calendario!$H$2:$H$53,"A")</f>
+        <f>SUMIFS(Calendario!$I$2:$I$52,Calendario!$G$2:$G$52,"Núcleo",Calendario!$H$2:$H$52,"A")</f>
         <v/>
       </c>
     </row>
@@ -629,7 +629,7 @@
         </is>
       </c>
       <c r="B17" s="7">
-        <f>SUMIFS(Calendario!$I$2:$I$53,Calendario!$G$2:$G$53,"Núcleo",Calendario!$H$2:$H$53,"B")</f>
+        <f>SUMIFS(Calendario!$I$2:$I$52,Calendario!$G$2:$G$52,"Núcleo",Calendario!$H$2:$H$52,"B")</f>
         <v/>
       </c>
     </row>
@@ -662,7 +662,7 @@
         </is>
       </c>
       <c r="B20" s="7">
-        <f>SUMIFS(Calendario!$I$2:$I$53,Calendario!$G$2:$G$53,"Fase B")</f>
+        <f>SUMIFS(Calendario!$I$2:$I$52,Calendario!$G$2:$G$52,"Fase B")</f>
         <v/>
       </c>
     </row>
@@ -759,7 +759,7 @@
         </is>
       </c>
       <c r="B32" s="7">
-        <f>SUMIFS(Calendario!$I$2:$I$53,Calendario!$G$2:$G$53,"Núcleo",Calendario!$B$2:$B$53,"&gt;="&amp;DATE(2026,10,1),Calendario!$B$2:$B$53,"&lt;"&amp;DATE(2026,11,1))</f>
+        <f>SUMIFS(Calendario!$I$2:$I$52,Calendario!$G$2:$G$52,"Núcleo",Calendario!$B$2:$B$52,"&gt;="&amp;DATE(2026,10,1),Calendario!$B$2:$B$52,"&lt;"&amp;DATE(2026,11,1))</f>
         <v/>
       </c>
     </row>
@@ -770,7 +770,7 @@
         </is>
       </c>
       <c r="B33" s="7">
-        <f>SUMIFS(Calendario!$I$2:$I$53,Calendario!$G$2:$G$53,"Núcleo",Calendario!$B$2:$B$53,"&gt;="&amp;DATE(2026,11,1),Calendario!$B$2:$B$53,"&lt;"&amp;DATE(2026,12,1))</f>
+        <f>SUMIFS(Calendario!$I$2:$I$52,Calendario!$G$2:$G$52,"Núcleo",Calendario!$B$2:$B$52,"&gt;="&amp;DATE(2026,11,1),Calendario!$B$2:$B$52,"&lt;"&amp;DATE(2026,12,1))</f>
         <v/>
       </c>
     </row>
@@ -781,7 +781,7 @@
         </is>
       </c>
       <c r="B34" s="7">
-        <f>SUMIFS(Calendario!$I$2:$I$53,Calendario!$G$2:$G$53,"Núcleo",Calendario!$B$2:$B$53,"&gt;="&amp;DATE(2026,12,1),Calendario!$B$2:$B$53,"&lt;"&amp;DATE(2027,1,1))</f>
+        <f>SUMIFS(Calendario!$I$2:$I$52,Calendario!$G$2:$G$52,"Núcleo",Calendario!$B$2:$B$52,"&gt;="&amp;DATE(2026,12,1),Calendario!$B$2:$B$52,"&lt;"&amp;DATE(2027,1,1))</f>
         <v/>
       </c>
     </row>
@@ -812,7 +812,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I35"/>
+  <dimension ref="A1:I34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -1272,15 +1272,15 @@
     <row r="11">
       <c r="A11" s="12" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>11</t>
         </is>
       </c>
       <c r="B11" s="13" t="n">
-        <v>46322</v>
+        <v>46324</v>
       </c>
       <c r="C11" s="14" t="inlineStr">
         <is>
-          <t>sáb 17 oct · taller</t>
+          <t>vie 16 oct · casa de Andrés</t>
         </is>
       </c>
       <c r="D11" s="14" t="inlineStr">
@@ -1290,7 +1290,7 @@
       </c>
       <c r="E11" s="14" t="inlineStr">
         <is>
-          <t>C1 · Cómo se pinta una pieza (1)</t>
+          <t>La casa se viste de Navidad</t>
         </is>
       </c>
       <c r="F11" s="14" t="inlineStr">
@@ -1305,7 +1305,7 @@
       </c>
       <c r="H11" s="14" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="I11" s="7">
@@ -1316,15 +1316,15 @@
     <row r="12">
       <c r="A12" s="12" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>12</t>
         </is>
       </c>
       <c r="B12" s="13" t="n">
-        <v>46324</v>
+        <v>46328</v>
       </c>
       <c r="C12" s="14" t="inlineStr">
         <is>
-          <t>vie 16 oct · casa de Andrés</t>
+          <t>vie 23 oct · tienda</t>
         </is>
       </c>
       <c r="D12" s="14" t="inlineStr">
@@ -1334,12 +1334,12 @@
       </c>
       <c r="E12" s="14" t="inlineStr">
         <is>
-          <t>La casa se viste de Navidad</t>
+          <t>C19 · Esta semana en la tienda (1)</t>
         </is>
       </c>
       <c r="F12" s="14" t="inlineStr">
         <is>
-          <t>Video</t>
+          <t>Historias</t>
         </is>
       </c>
       <c r="G12" s="14" t="inlineStr">
@@ -1349,7 +1349,7 @@
       </c>
       <c r="H12" s="14" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="I12" s="7">
@@ -1360,15 +1360,15 @@
     <row r="13">
       <c r="A13" s="12" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>13</t>
         </is>
       </c>
       <c r="B13" s="13" t="n">
-        <v>46328</v>
+        <v>46329</v>
       </c>
       <c r="C13" s="14" t="inlineStr">
         <is>
-          <t>vie 23 oct · tienda</t>
+          <t>vie 16 oct · casa de Andrés</t>
         </is>
       </c>
       <c r="D13" s="14" t="inlineStr">
@@ -1378,12 +1378,12 @@
       </c>
       <c r="E13" s="14" t="inlineStr">
         <is>
-          <t>C19 · Esta semana en la tienda (1)</t>
+          <t>Drop 1 · Flores</t>
         </is>
       </c>
       <c r="F13" s="14" t="inlineStr">
         <is>
-          <t>Historias</t>
+          <t>Video</t>
         </is>
       </c>
       <c r="G13" s="14" t="inlineStr">
@@ -1393,7 +1393,7 @@
       </c>
       <c r="H13" s="14" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="I13" s="7">
@@ -1404,11 +1404,11 @@
     <row r="14">
       <c r="A14" s="12" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>15</t>
         </is>
       </c>
       <c r="B14" s="13" t="n">
-        <v>46329</v>
+        <v>46333</v>
       </c>
       <c r="C14" s="14" t="inlineStr">
         <is>
@@ -1422,12 +1422,12 @@
       </c>
       <c r="E14" s="14" t="inlineStr">
         <is>
-          <t>Drop 1 · Flores</t>
+          <t>C11 · Cómo vestir una mesa por capas</t>
         </is>
       </c>
       <c r="F14" s="14" t="inlineStr">
         <is>
-          <t>Video</t>
+          <t>Carrusel</t>
         </is>
       </c>
       <c r="G14" s="14" t="inlineStr">
@@ -1437,7 +1437,7 @@
       </c>
       <c r="H14" s="14" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="I14" s="7">
@@ -1448,15 +1448,15 @@
     <row r="15">
       <c r="A15" s="12" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>16</t>
         </is>
       </c>
       <c r="B15" s="13" t="n">
-        <v>46331</v>
+        <v>46336</v>
       </c>
       <c r="C15" s="14" t="inlineStr">
         <is>
-          <t>mar 3 nov · casa o tienda</t>
+          <t>vie 16 oct · casa de Andrés</t>
         </is>
       </c>
       <c r="D15" s="14" t="inlineStr">
@@ -1466,7 +1466,7 @@
       </c>
       <c r="E15" s="14" t="inlineStr">
         <is>
-          <t>C10 · Pon la mesa con tus piezas pintadas</t>
+          <t>Drop 2 · Caballos a cuadros</t>
         </is>
       </c>
       <c r="F15" s="14" t="inlineStr">
@@ -1481,7 +1481,7 @@
       </c>
       <c r="H15" s="14" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="I15" s="7">
@@ -1492,25 +1492,25 @@
     <row r="16">
       <c r="A16" s="12" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>17</t>
         </is>
       </c>
       <c r="B16" s="13" t="n">
-        <v>46333</v>
+        <v>46338</v>
       </c>
       <c r="C16" s="14" t="inlineStr">
         <is>
-          <t>vie 16 oct · casa de Andrés</t>
+          <t>lun 5 oct · atelier</t>
         </is>
       </c>
       <c r="D16" s="14" t="inlineStr">
         <is>
-          <t>Alado &amp; Co.</t>
+          <t>Bride</t>
         </is>
       </c>
       <c r="E16" s="14" t="inlineStr">
         <is>
-          <t>C11 · Cómo vestir una mesa por capas</t>
+          <t>B11 · Del primer lápiz a la entrega</t>
         </is>
       </c>
       <c r="F16" s="14" t="inlineStr">
@@ -1536,15 +1536,15 @@
     <row r="17">
       <c r="A17" s="12" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>18</t>
         </is>
       </c>
       <c r="B17" s="13" t="n">
-        <v>46336</v>
+        <v>46342</v>
       </c>
       <c r="C17" s="14" t="inlineStr">
         <is>
-          <t>vie 16 oct · casa de Andrés</t>
+          <t>vie 6 nov · tienda</t>
         </is>
       </c>
       <c r="D17" s="14" t="inlineStr">
@@ -1554,12 +1554,12 @@
       </c>
       <c r="E17" s="14" t="inlineStr">
         <is>
-          <t>Drop 2 · Caballos a cuadros</t>
+          <t>C19 · Esta semana en la tienda (2)</t>
         </is>
       </c>
       <c r="F17" s="14" t="inlineStr">
         <is>
-          <t>Video</t>
+          <t>Historias</t>
         </is>
       </c>
       <c r="G17" s="14" t="inlineStr">
@@ -1569,7 +1569,7 @@
       </c>
       <c r="H17" s="14" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="I17" s="7">
@@ -1580,30 +1580,30 @@
     <row r="18">
       <c r="A18" s="12" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>19</t>
         </is>
       </c>
       <c r="B18" s="13" t="n">
-        <v>46338</v>
+        <v>46343</v>
       </c>
       <c r="C18" s="14" t="inlineStr">
         <is>
-          <t>lun 5 oct · atelier</t>
+          <t>vie 16 oct · casa de Andrés</t>
         </is>
       </c>
       <c r="D18" s="14" t="inlineStr">
         <is>
-          <t>Bride</t>
+          <t>Alado &amp; Co.</t>
         </is>
       </c>
       <c r="E18" s="14" t="inlineStr">
         <is>
-          <t>B11 · Del primer lápiz a la entrega</t>
+          <t>Drop 3 · Ángeles y ciervos</t>
         </is>
       </c>
       <c r="F18" s="14" t="inlineStr">
         <is>
-          <t>Carrusel</t>
+          <t>Video</t>
         </is>
       </c>
       <c r="G18" s="14" t="inlineStr">
@@ -1613,7 +1613,7 @@
       </c>
       <c r="H18" s="14" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="I18" s="7">
@@ -1624,30 +1624,30 @@
     <row r="19">
       <c r="A19" s="12" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>20</t>
         </is>
       </c>
       <c r="B19" s="13" t="n">
-        <v>46342</v>
+        <v>46345</v>
       </c>
       <c r="C19" s="14" t="inlineStr">
         <is>
-          <t>vie 6 nov · tienda</t>
+          <t>lun 5 oct · atelier</t>
         </is>
       </c>
       <c r="D19" s="14" t="inlineStr">
         <is>
-          <t>Alado &amp; Co.</t>
+          <t>Celebration</t>
         </is>
       </c>
       <c r="E19" s="14" t="inlineStr">
         <is>
-          <t>C19 · Esta semana en la tienda (2)</t>
+          <t>B15 · Prom y 15s: tu vestido, único</t>
         </is>
       </c>
       <c r="F19" s="14" t="inlineStr">
         <is>
-          <t>Historias</t>
+          <t>Carrusel</t>
         </is>
       </c>
       <c r="G19" s="14" t="inlineStr">
@@ -1657,7 +1657,7 @@
       </c>
       <c r="H19" s="14" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="I19" s="7">
@@ -1668,15 +1668,15 @@
     <row r="20">
       <c r="A20" s="12" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>21</t>
         </is>
       </c>
       <c r="B20" s="13" t="n">
-        <v>46343</v>
+        <v>46347</v>
       </c>
       <c r="C20" s="14" t="inlineStr">
         <is>
-          <t>vie 16 oct · casa de Andrés</t>
+          <t>jue 12 nov · casa de Andrés</t>
         </is>
       </c>
       <c r="D20" s="14" t="inlineStr">
@@ -1686,7 +1686,7 @@
       </c>
       <c r="E20" s="14" t="inlineStr">
         <is>
-          <t>Drop 3 · Ángeles y ciervos</t>
+          <t>Receta de Navidad en la mesa Alado</t>
         </is>
       </c>
       <c r="F20" s="14" t="inlineStr">
@@ -1701,7 +1701,7 @@
       </c>
       <c r="H20" s="14" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="I20" s="7">
@@ -1712,30 +1712,30 @@
     <row r="21">
       <c r="A21" s="12" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>22</t>
         </is>
       </c>
       <c r="B21" s="13" t="n">
-        <v>46345</v>
+        <v>46349</v>
       </c>
       <c r="C21" s="14" t="inlineStr">
         <is>
-          <t>lun 5 oct · atelier</t>
+          <t>mar 17 nov · Alejo</t>
         </is>
       </c>
       <c r="D21" s="14" t="inlineStr">
         <is>
-          <t>Celebration</t>
+          <t>Bride</t>
         </is>
       </c>
       <c r="E21" s="14" t="inlineStr">
         <is>
-          <t>B15 · Prom y 15s: tu vestido, único</t>
+          <t>B17 · Caja de preguntas con Alejo</t>
         </is>
       </c>
       <c r="F21" s="14" t="inlineStr">
         <is>
-          <t>Carrusel</t>
+          <t>Historias</t>
         </is>
       </c>
       <c r="G21" s="14" t="inlineStr">
@@ -1745,7 +1745,7 @@
       </c>
       <c r="H21" s="14" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="I21" s="7">
@@ -1756,25 +1756,25 @@
     <row r="22">
       <c r="A22" s="12" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>23</t>
         </is>
       </c>
       <c r="B22" s="13" t="n">
-        <v>46347</v>
+        <v>46350</v>
       </c>
       <c r="C22" s="14" t="inlineStr">
         <is>
-          <t>jue 12 nov · casa de Andrés</t>
+          <t>mar 17 nov · Alejo</t>
         </is>
       </c>
       <c r="D22" s="14" t="inlineStr">
         <is>
-          <t>Alado &amp; Co.</t>
+          <t>Bride</t>
         </is>
       </c>
       <c r="E22" s="14" t="inlineStr">
         <is>
-          <t>Receta de Navidad en la mesa Alado</t>
+          <t>B3 · Notas de Alejo (manuscritas)</t>
         </is>
       </c>
       <c r="F22" s="14" t="inlineStr">
@@ -1789,7 +1789,7 @@
       </c>
       <c r="H22" s="14" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="I22" s="7">
@@ -1800,30 +1800,30 @@
     <row r="23">
       <c r="A23" s="12" t="inlineStr">
         <is>
-          <t>22</t>
+          <t>24</t>
         </is>
       </c>
       <c r="B23" s="13" t="n">
-        <v>46349</v>
+        <v>46352</v>
       </c>
       <c r="C23" s="14" t="inlineStr">
         <is>
-          <t>mar 17 nov · Alejo</t>
+          <t>jue 19 nov · tienda</t>
         </is>
       </c>
       <c r="D23" s="14" t="inlineStr">
         <is>
-          <t>Bride</t>
+          <t>Alado &amp; Co.</t>
         </is>
       </c>
       <c r="E23" s="14" t="inlineStr">
         <is>
-          <t>B17 · Caja de preguntas con Alejo</t>
+          <t>Armamos una ancheta Alado</t>
         </is>
       </c>
       <c r="F23" s="14" t="inlineStr">
         <is>
-          <t>Historias</t>
+          <t>Video</t>
         </is>
       </c>
       <c r="G23" s="14" t="inlineStr">
@@ -1844,30 +1844,30 @@
     <row r="24">
       <c r="A24" s="12" t="inlineStr">
         <is>
-          <t>23</t>
+          <t>25</t>
         </is>
       </c>
       <c r="B24" s="13" t="n">
-        <v>46350</v>
+        <v>46354</v>
       </c>
       <c r="C24" s="14" t="inlineStr">
         <is>
-          <t>mar 17 nov · Alejo</t>
+          <t>sáb 21 nov · El Retiro</t>
         </is>
       </c>
       <c r="D24" s="14" t="inlineStr">
         <is>
-          <t>Bride</t>
+          <t>Alado &amp; Co.</t>
         </is>
       </c>
       <c r="E24" s="14" t="inlineStr">
         <is>
-          <t>B3 · Notas de Alejo (manuscritas)</t>
+          <t>C14 · Un día en El Retiro en Navidad</t>
         </is>
       </c>
       <c r="F24" s="14" t="inlineStr">
         <is>
-          <t>Video</t>
+          <t>Carrusel</t>
         </is>
       </c>
       <c r="G24" s="14" t="inlineStr">
@@ -1877,7 +1877,7 @@
       </c>
       <c r="H24" s="14" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="I24" s="7">
@@ -1888,30 +1888,30 @@
     <row r="25">
       <c r="A25" s="12" t="inlineStr">
         <is>
-          <t>24</t>
+          <t>26</t>
         </is>
       </c>
       <c r="B25" s="13" t="n">
-        <v>46352</v>
+        <v>46356</v>
       </c>
       <c r="C25" s="14" t="inlineStr">
         <is>
-          <t>jue 19 nov · tienda</t>
+          <t>mar 17 nov · Alejo</t>
         </is>
       </c>
       <c r="D25" s="14" t="inlineStr">
         <is>
-          <t>Alado &amp; Co.</t>
+          <t>Bride</t>
         </is>
       </c>
       <c r="E25" s="14" t="inlineStr">
         <is>
-          <t>Armamos una ancheta Alado</t>
+          <t>B20 · Agenda abierta hasta el 11 de diciembre</t>
         </is>
       </c>
       <c r="F25" s="14" t="inlineStr">
         <is>
-          <t>Video</t>
+          <t>Historias</t>
         </is>
       </c>
       <c r="G25" s="14" t="inlineStr">
@@ -1921,7 +1921,7 @@
       </c>
       <c r="H25" s="14" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="I25" s="7">
@@ -1932,15 +1932,15 @@
     <row r="26">
       <c r="A26" s="12" t="inlineStr">
         <is>
-          <t>25</t>
+          <t>27</t>
         </is>
       </c>
       <c r="B26" s="13" t="n">
-        <v>46354</v>
+        <v>46305</v>
       </c>
       <c r="C26" s="14" t="inlineStr">
         <is>
-          <t>sáb 21 nov · El Retiro</t>
+          <t>mar 6 oct · pre-taller</t>
         </is>
       </c>
       <c r="D26" s="14" t="inlineStr">
@@ -1950,7 +1950,7 @@
       </c>
       <c r="E26" s="14" t="inlineStr">
         <is>
-          <t>C14 · Un día en El Retiro en Navidad</t>
+          <t>Cómo participar en el taller de cerámica</t>
         </is>
       </c>
       <c r="F26" s="14" t="inlineStr">
@@ -1965,7 +1965,7 @@
       </c>
       <c r="H26" s="14" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="I26" s="7">
@@ -1976,35 +1976,35 @@
     <row r="27">
       <c r="A27" s="12" t="inlineStr">
         <is>
-          <t>26</t>
+          <t>V1</t>
         </is>
       </c>
       <c r="B27" s="13" t="n">
-        <v>46356</v>
+        <v>46371</v>
       </c>
       <c r="C27" s="14" t="inlineStr">
         <is>
-          <t>mar 17 nov · Alejo</t>
+          <t>1–9 dic · banco</t>
         </is>
       </c>
       <c r="D27" s="14" t="inlineStr">
         <is>
-          <t>Bride</t>
+          <t>Alado &amp; Co.</t>
         </is>
       </c>
       <c r="E27" s="14" t="inlineStr">
         <is>
-          <t>B20 · Agenda abierta hasta el 11 de diciembre</t>
+          <t>No es solo Navidad (flores y caballos todo el año)</t>
         </is>
       </c>
       <c r="F27" s="14" t="inlineStr">
         <is>
-          <t>Historias</t>
+          <t>Video</t>
         </is>
       </c>
       <c r="G27" s="14" t="inlineStr">
         <is>
-          <t>Núcleo</t>
+          <t>Fase B</t>
         </is>
       </c>
       <c r="H27" s="14" t="inlineStr">
@@ -2020,11 +2020,11 @@
     <row r="28">
       <c r="A28" s="12" t="inlineStr">
         <is>
-          <t>V1</t>
+          <t>V2</t>
         </is>
       </c>
       <c r="B28" s="13" t="n">
-        <v>46371</v>
+        <v>46374</v>
       </c>
       <c r="C28" s="14" t="inlineStr">
         <is>
@@ -2033,12 +2033,12 @@
       </c>
       <c r="D28" s="14" t="inlineStr">
         <is>
-          <t>Alado &amp; Co.</t>
+          <t>Alado</t>
         </is>
       </c>
       <c r="E28" s="14" t="inlineStr">
         <is>
-          <t>No es solo Navidad (flores y caballos todo el año)</t>
+          <t>Regala Alado (envolver)</t>
         </is>
       </c>
       <c r="F28" s="14" t="inlineStr">
@@ -2064,11 +2064,11 @@
     <row r="29">
       <c r="A29" s="12" t="inlineStr">
         <is>
-          <t>V2</t>
+          <t>V3</t>
         </is>
       </c>
       <c r="B29" s="13" t="n">
-        <v>46374</v>
+        <v>46378</v>
       </c>
       <c r="C29" s="14" t="inlineStr">
         <is>
@@ -2077,12 +2077,12 @@
       </c>
       <c r="D29" s="14" t="inlineStr">
         <is>
-          <t>Alado</t>
+          <t>Alado &amp; Co.</t>
         </is>
       </c>
       <c r="E29" s="14" t="inlineStr">
         <is>
-          <t>Regala Alado (envolver)</t>
+          <t>Cómo montar una mesa que se recuerde</t>
         </is>
       </c>
       <c r="F29" s="14" t="inlineStr">
@@ -2108,11 +2108,11 @@
     <row r="30">
       <c r="A30" s="12" t="inlineStr">
         <is>
-          <t>V3</t>
+          <t>V4</t>
         </is>
       </c>
       <c r="B30" s="13" t="n">
-        <v>46378</v>
+        <v>46385</v>
       </c>
       <c r="C30" s="14" t="inlineStr">
         <is>
@@ -2126,7 +2126,7 @@
       </c>
       <c r="E30" s="14" t="inlineStr">
         <is>
-          <t>Cómo montar una mesa que se recuerde</t>
+          <t>Cómo se pinta una pieza</t>
         </is>
       </c>
       <c r="F30" s="14" t="inlineStr">
@@ -2152,11 +2152,11 @@
     <row r="31">
       <c r="A31" s="12" t="inlineStr">
         <is>
-          <t>V4</t>
+          <t>V5</t>
         </is>
       </c>
       <c r="B31" s="13" t="n">
-        <v>46385</v>
+        <v>46392</v>
       </c>
       <c r="C31" s="14" t="inlineStr">
         <is>
@@ -2165,17 +2165,17 @@
       </c>
       <c r="D31" s="14" t="inlineStr">
         <is>
-          <t>Alado &amp; Co.</t>
+          <t>Bride</t>
         </is>
       </c>
       <c r="E31" s="14" t="inlineStr">
         <is>
-          <t>C1 · Cómo se pinta una pieza (2)</t>
+          <t>Notas de Alejo: novias 2027</t>
         </is>
       </c>
       <c r="F31" s="14" t="inlineStr">
         <is>
-          <t>Video</t>
+          <t>Carrusel</t>
         </is>
       </c>
       <c r="G31" s="14" t="inlineStr">
@@ -2196,11 +2196,11 @@
     <row r="32">
       <c r="A32" s="12" t="inlineStr">
         <is>
-          <t>V5</t>
+          <t>V6</t>
         </is>
       </c>
       <c r="B32" s="13" t="n">
-        <v>46392</v>
+        <v>46396</v>
       </c>
       <c r="C32" s="14" t="inlineStr">
         <is>
@@ -2214,7 +2214,7 @@
       </c>
       <c r="E32" s="14" t="inlineStr">
         <is>
-          <t>Notas de Alejo: novias 2027</t>
+          <t>Cómo agendar tu cita desde el 12 de enero</t>
         </is>
       </c>
       <c r="F32" s="14" t="inlineStr">
@@ -2237,52 +2237,8 @@
         <v/>
       </c>
     </row>
-    <row r="33">
-      <c r="A33" s="12" t="inlineStr">
-        <is>
-          <t>V6</t>
-        </is>
-      </c>
-      <c r="B33" s="13" t="n">
-        <v>46396</v>
-      </c>
-      <c r="C33" s="14" t="inlineStr">
-        <is>
-          <t>1–9 dic · banco</t>
-        </is>
-      </c>
-      <c r="D33" s="14" t="inlineStr">
-        <is>
-          <t>Bride</t>
-        </is>
-      </c>
-      <c r="E33" s="14" t="inlineStr">
-        <is>
-          <t>Cómo agendar tu cita desde el 12 de enero</t>
-        </is>
-      </c>
-      <c r="F33" s="14" t="inlineStr">
-        <is>
-          <t>Carrusel</t>
-        </is>
-      </c>
-      <c r="G33" s="14" t="inlineStr">
-        <is>
-          <t>Fase B</t>
-        </is>
-      </c>
-      <c r="H33" s="14" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="I33" s="7">
-        <f>IF(F33="Video",Presupuesto!$B$5,IF(F33="Carrusel",Presupuesto!$B$6,IF(F33="Historias",Presupuesto!$B$7,0)))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="35">
-      <c r="E35" s="2" t="inlineStr">
+    <row r="34">
+      <c r="E34" s="2" t="inlineStr">
         <is>
           <t>Cambia fecha, formato, fase o prioridad y el presupuesto se recalcula solo.</t>
         </is>
@@ -2290,13 +2246,13 @@
     </row>
   </sheetData>
   <dataValidations count="3">
-    <dataValidation sqref="F2:F53" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="F2:F52" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Video,Carrusel,Historias"</formula1>
     </dataValidation>
-    <dataValidation sqref="G2:G53" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="G2:G52" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Núcleo,Fase B"</formula1>
     </dataValidation>
-    <dataValidation sqref="H2:H53" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="H2:H52" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"A,B"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>